<commit_message>
Fix combined-1000 workbook to use the actual committed 300, not a stale upload
The Original_300 section was built from a later re-uploaded reference file
that differed from the repo's own arabic_english_codeswitching_300.csv in
~50 rows (shorter wording). The committed 300 file itself was never
modified -- only the combined workbook pulled from the wrong source.
Now rebuilt directly from arabic_english_codeswitching_300.csv so the
first 300 rows match it exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155UPXv8Dk7askKg634TkFB
</commit_message>
<xml_diff>
--- a/arabic_english_codeswitching_1000_combined.xlsx
+++ b/arabic_english_codeswitching_1000_combined.xlsx
@@ -451,12 +451,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>حدثت الـ API اليوم.</t>
+          <t>حدثت الـ API اليوم واختبرت كل الـ endpoints.</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>API, endpoints</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -468,12 +468,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>رفعت المشروع على GitHub.</t>
+          <t>رفعت المشروع على GitHub وسويت commit جديد.</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>GitHub, commit</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>استخدمت USB جديداً.</t>
+          <t>استخدمت USB جديد عشان أنقل الملفات.</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -502,7 +502,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>جربت الـ LLM على بيانات جديدة.</t>
+          <t>جربت الـ LLM على بيانات جديدة وطلعت النتيجة ممتازة.</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -519,7 +519,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>فتحت الـ dashboard وشفت النتائج.</t>
+          <t>فتحت الـ dashboard وشفت النتائج بسرعة.</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>سويت deploy للتطبيق على الـ server.</t>
+          <t>سويت deploy للتطبيق على الـ server قبل شوي.</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>سجلت دخولي عن طريق SSO.</t>
+          <t>سجلت دخولي عن طريق SSO عشان أوفر وقت.</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -570,7 +570,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>حملت الـ update من الـ App Store.</t>
+          <t>حملت الـ update من الـ App Store الليلة.</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>شغّلت الـ WiFi وربطت الـ laptop.</t>
+          <t>شغّلت الـ WiFi وربطت الـ laptop بسرعة.</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -604,7 +604,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>استخدمنا Slack للتواصل بين الفريق.</t>
+          <t>استخدمنا Slack للتواصل بين الفريق طول اليوم.</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -621,7 +621,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>عملنا merge للـ branch في Git.</t>
+          <t>عملنا merge للـ branch في Git بعد المراجعة.</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>فتحت ticket في Jira.</t>
+          <t>فتحت ticket في Jira عشان أبلغ عن المشكلة.</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -655,7 +655,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>شفت error في الـ log file.</t>
+          <t>شفت error في الـ log file وقفلت السيرفر.</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -672,7 +672,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>سويت backup للـ database.</t>
+          <t>سويت backup للـ database قبل التحديث.</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -689,7 +689,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>رجّعت الـ settings للوضع الافتراضي.</t>
+          <t>رجّعت الـ settings للوضع الافتراضي بعد المشكلة.</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -706,7 +706,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>استخدمت ChatGPT لمراجعة النص.</t>
+          <t>استخدمت ChatGPT لمراجعة النص قبل الإرسال.</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -723,7 +723,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>شغّلت الـ VPN قبل الدخول.</t>
+          <t>شغّلت الـ VPN قبل الدخول على الشبكة.</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ربطت الـ Bluetooth بالـ speaker.</t>
+          <t>ربطت الـ Bluetooth بالـ speaker وشغلت الأغنية.</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>سويت debug للكود عشان أعرف مصدر المشكلة.</t>
+          <t>سويت debug للكود عشان ألقى مصدر المشكلة.</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -978,7 +978,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>سوينا setup لبيئة العمل على الـ cloud.</t>
+          <t>عملنا setup لبيئة العمل على الـ cloud.</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>لازم نسوي refactor للكود عشان يصير أنظف.</t>
+          <t>لازم نعمل refactor للكود عشان يصير أنظف.</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1216,12 +1216,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>نزلت story جديدة على الـ Snapchat الصبح.</t>
+          <t>نزلت story جديدة على الـ Instagram الصبح.</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>story, Snapchat</t>
+          <t>story, Instagram</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -1250,7 +1250,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>سويت repost للـ tweet اللي عجبني.</t>
+          <t>عملت repost للـ tweet اللي عجبني.</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1318,12 +1318,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>سويت live على Instagram وتفاعل الناس زين.</t>
+          <t>سويت live على Snapchat وتفاعل الناس زين.</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>live, Instagram</t>
+          <t>live, Snapchat</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -1335,7 +1335,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>الـ reels جتها views كثير بليلة وحدة.</t>
+          <t>الريلز حصلت views كثير بليلة وحدة.</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>سويت block لحساب مزعج على X.</t>
+          <t>عملت block لحساب مزعج على X.</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>سويت share للملف في الـ group.</t>
+          <t>عملت share للمنشور في الـ group.</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1420,7 +1420,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>اكتشفت ان الـ algorithm تفضل الفيديوهات القصيرة.</t>
+          <t>الخوارزمية algorithm تفضل الفيديوهات القصيرة.</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -1454,7 +1454,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>الحساب صار له suspend بدون سبب واضح، للأسف!</t>
+          <t>الحساب انعمله suspend بدون سبب واضح، للأسف!</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1471,7 +1471,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>نزلت reel وكتبت caption يضحك.</t>
+          <t>نزلت reel وحطيت caption مضحك.</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>الـ comments حقت البوست كلها إيجابية.</t>
+          <t>الـ comments تحت البوست كلها إيجابية.</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>سويت follow للحساب الجديد اللي فتحوه.</t>
+          <t>عملت follow للحساب الجديد اللي فتحوه.</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>سويت subscribe لقناته الجديدة على YouTube.</t>
+          <t>عملت subscribe لقناته الجديدة على YouTube.</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -2100,7 +2100,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>سويت attach للملف قبل ما أرسل الإيميل.</t>
+          <t>عملت attach للملف قبل ما أرسل الإيميل.</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2270,7 +2270,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>سويت approve على الطلب المالي.</t>
+          <t>عملت approve على الطلب المالي.</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -2950,7 +2950,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>سويت sync بين الجوال واللابتوب.</t>
+          <t>عملت sync بين الجوال واللابتوب.</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -3494,7 +3494,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>سويت subscription شهري لتطبيق التمارين.</t>
+          <t>عملت subscription شهري لتطبيق التمارين.</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -3919,7 +3919,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>سويت check-in مبكر عن طريق التطبيق.</t>
+          <t>عملت check-in مبكر عن طريق التطبيق.</t>
         </is>
       </c>
       <c r="B206" s="3" t="inlineStr">
@@ -4344,7 +4344,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>سويت refund للطلب لأنه تأخر كثير.</t>
+          <t>عملت refund للطلب لأنه تأخر كثير.</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr">
@@ -4463,7 +4463,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>سويت compare بين سعر المتجر والمتجر المنافس.</t>
+          <t>عملت compare بين سعر المتجر والمتجر المنافس.</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
@@ -4599,7 +4599,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>سويت order من تطبيق Jarir للأدوات المكتبية.</t>
+          <t>عملت order من تطبيق Jarir للأدوات المكتبية.</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr">
@@ -4854,7 +4854,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>سويت install للتطبيق وواجهت مشكلة.</t>
+          <t>عملت install للتطبيق وواجهت مشكلة.</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr">
@@ -4905,7 +4905,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>سويت update للتطبيق عشان أحل المشكلة.</t>
+          <t>عملت update للتطبيق عشان أحل المشكلة.</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
@@ -4990,7 +4990,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>سويت mute لمجموعة الواتساب المزعجة.</t>
+          <t>عملت mute لمجموعة الواتساب المزعجة.</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>سويت forward للرسالة لصديقي.</t>
+          <t>عملت forward للرسالة لصديقي.</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>سويت clear للـ cache عشان يشتغل أسرع.</t>
+          <t>عملت clear للـ cache عشان يشتغل أسرع.</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr">
@@ -5279,7 +5279,7 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>سويت restart سريع للجوال بعد ما تعلق.</t>
+          <t>عملت restart سريع للجوال بعد ما تعلق.</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
@@ -5347,7 +5347,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>سويت verify لرقمي بعد ما نزلت التطبيق.</t>
+          <t>عملت verify لرقمي بعد ما نزلت التطبيق.</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
@@ -5432,7 +5432,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>سويت report لحساب مزيف يتصل بالناس.</t>
+          <t>عملت report لحساب مزيف يتصل بالناس.</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
@@ -5500,7 +5500,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>سويت transfer للملفات بين الجوالين بسرعة.</t>
+          <t>عملت transfer للملفات بين الجوالين بسرعة.</t>
         </is>
       </c>
       <c r="B299" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Compute Word_Frequency for the original 300 too (text left untouched)
Previously the original 300 rows had a blank Word_Frequency. Now every
row in the combined 1000 gets a running per-word count in sheet order
(300 first, then 700) -- sentence text and English_Terms for the
original 300 remain byte-identical to arabic_english_codeswitching_300.csv.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155UPXv8Dk7askKg634TkFB
</commit_message>
<xml_diff>
--- a/arabic_english_codeswitching_1000_combined.xlsx
+++ b/arabic_english_codeswitching_1000_combined.xlsx
@@ -428,7 +428,7 @@
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -465,7 +465,11 @@
           <t>API, endpoints</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>API(1), endpoints(1)</t>
+        </is>
+      </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -483,7 +487,11 @@
           <t>GitHub, commit</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>GitHub(1), commit(1)</t>
+        </is>
+      </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -501,7 +509,11 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>USB(1)</t>
+        </is>
+      </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -519,7 +531,11 @@
           <t>LLM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>LLM(1)</t>
+        </is>
+      </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -537,7 +553,11 @@
           <t>dashboard</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>dashboard(1)</t>
+        </is>
+      </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -555,7 +575,11 @@
           <t>deploy, server</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>deploy(1), server(1)</t>
+        </is>
+      </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -573,7 +597,11 @@
           <t>SSO</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>SSO(1)</t>
+        </is>
+      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -591,7 +619,11 @@
           <t>update, App Store</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>update(1), App(1), Store(1)</t>
+        </is>
+      </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -609,7 +641,11 @@
           <t>WiFi, laptop</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>WiFi(1), laptop(1)</t>
+        </is>
+      </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -627,7 +663,11 @@
           <t>Slack</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Slack(1)</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -645,7 +685,11 @@
           <t>merge, branch, Git</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>merge(1), branch(1), Git(1)</t>
+        </is>
+      </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -663,7 +707,11 @@
           <t>ticket, Jira</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>ticket(1), Jira(1)</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -681,7 +729,11 @@
           <t>error, log file</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>error(1), log(1), file(1)</t>
+        </is>
+      </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -699,7 +751,11 @@
           <t>backup, database</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>backup(1), database(1)</t>
+        </is>
+      </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -717,7 +773,11 @@
           <t>settings</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>settings(1)</t>
+        </is>
+      </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -735,7 +795,11 @@
           <t>ChatGPT</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ChatGPT(1)</t>
+        </is>
+      </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -753,7 +817,11 @@
           <t>VPN</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>VPN(1)</t>
+        </is>
+      </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -771,7 +839,11 @@
           <t>Bluetooth, speaker</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Bluetooth(1), speaker(1)</t>
+        </is>
+      </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -789,7 +861,11 @@
           <t>code review, pull request</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>code(1), review(1), pull(1), request(1)</t>
+        </is>
+      </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -807,7 +883,11 @@
           <t>bug, production</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>bug(1), production(1)</t>
+        </is>
+      </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -825,7 +905,11 @@
           <t>token, environment variables</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>token(1), environment(1), variables(1)</t>
+        </is>
+      </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -843,7 +927,11 @@
           <t>backend, frontend</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr"/>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>backend(1), frontend(1)</t>
+        </is>
+      </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -861,7 +949,11 @@
           <t>push, CI</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>push(1), CI(1)</t>
+        </is>
+      </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -879,7 +971,11 @@
           <t>query, optimize</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>query(1), optimize(1)</t>
+        </is>
+      </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -897,7 +993,11 @@
           <t>terminal, script</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>terminal(1), script(1)</t>
+        </is>
+      </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -915,7 +1015,11 @@
           <t>test, feature</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>test(1), feature(1)</t>
+        </is>
+      </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -933,7 +1037,11 @@
           <t>container, Docker</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>container(1), Docker(1)</t>
+        </is>
+      </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -951,7 +1059,11 @@
           <t>build, staging, production</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr"/>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>build(1), staging(1), production(2)</t>
+        </is>
+      </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -969,7 +1081,11 @@
           <t>debug</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>debug(1)</t>
+        </is>
+      </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -987,7 +1103,11 @@
           <t>API, response</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>API(2), response(1)</t>
+        </is>
+      </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1005,7 +1125,11 @@
           <t>Notion, documentation</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Notion(1), documentation(1)</t>
+        </is>
+      </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1023,7 +1147,11 @@
           <t>setup, cloud</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>setup(1), cloud(1)</t>
+        </is>
+      </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1041,7 +1169,11 @@
           <t>pipeline, config</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>pipeline(1), config(1)</t>
+        </is>
+      </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1059,7 +1191,11 @@
           <t>dependencies</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>dependencies(1)</t>
+        </is>
+      </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1077,7 +1213,11 @@
           <t>clone, repository</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>clone(1), repository(1)</t>
+        </is>
+      </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1095,7 +1235,11 @@
           <t>function, null</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>function(1), null(1)</t>
+        </is>
+      </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1113,7 +1257,11 @@
           <t>Agile, sprint</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Agile(1), sprint(1)</t>
+        </is>
+      </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1131,7 +1279,11 @@
           <t>frontend, backend, REST API</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>frontend(2), backend(2), REST(1), API(3)</t>
+        </is>
+      </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1149,7 +1301,11 @@
           <t>refactor</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>refactor(1)</t>
+        </is>
+      </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1167,7 +1323,11 @@
           <t>commit</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>commit(2)</t>
+        </is>
+      </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1185,7 +1345,11 @@
           <t>standup</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>standup(1)</t>
+        </is>
+      </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1203,7 +1367,11 @@
           <t>caching</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr"/>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>caching(1)</t>
+        </is>
+      </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1221,7 +1389,11 @@
           <t>conflict, merge</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>conflict(1), merge(2)</t>
+        </is>
+      </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1239,7 +1411,11 @@
           <t>Postman, API</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Postman(1), API(4)</t>
+        </is>
+      </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1257,7 +1433,11 @@
           <t>migration, database</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>migration(1), database(2)</t>
+        </is>
+      </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1275,7 +1455,11 @@
           <t>story, Instagram</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>story(1), Instagram(1)</t>
+        </is>
+      </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1293,7 +1477,11 @@
           <t>trending, TikTok</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>trending(1), TikTok(1)</t>
+        </is>
+      </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1311,7 +1499,11 @@
           <t>repost, tweet</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>repost(1), tweet(1)</t>
+        </is>
+      </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1329,7 +1521,11 @@
           <t>followers, collab</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr"/>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>followers(1), collab(1)</t>
+        </is>
+      </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1347,7 +1543,11 @@
           <t>hashtag</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr"/>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>hashtag(1)</t>
+        </is>
+      </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1365,7 +1565,11 @@
           <t>verified</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>verified(1)</t>
+        </is>
+      </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1383,7 +1587,11 @@
           <t>live, Snapchat</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr"/>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>live(1), Snapchat(1)</t>
+        </is>
+      </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1401,7 +1609,11 @@
           <t>reels, views</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr"/>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>reels(1), views(1)</t>
+        </is>
+      </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1419,7 +1631,11 @@
           <t>block, X</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>block(1), X(1)</t>
+        </is>
+      </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1437,7 +1653,11 @@
           <t>engagement</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>engagement(1)</t>
+        </is>
+      </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1455,7 +1675,11 @@
           <t>highlight</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>highlight(1)</t>
+        </is>
+      </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1473,7 +1697,11 @@
           <t>share, group</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>share(1), group(1)</t>
+        </is>
+      </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1491,7 +1719,11 @@
           <t>algorithm</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr"/>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>algorithm(1)</t>
+        </is>
+      </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1509,7 +1741,11 @@
           <t>poll, story</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr"/>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>poll(1), story(2)</t>
+        </is>
+      </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1527,7 +1763,11 @@
           <t>suspend</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr"/>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>suspend(1)</t>
+        </is>
+      </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1545,7 +1785,11 @@
           <t>reel, caption</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>reel(1), caption(1)</t>
+        </is>
+      </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1563,7 +1807,11 @@
           <t>comments</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr"/>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>comments(1)</t>
+        </is>
+      </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1581,7 +1829,11 @@
           <t>follow</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>follow(1)</t>
+        </is>
+      </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1599,7 +1851,11 @@
           <t>trend</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>trend(1)</t>
+        </is>
+      </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1617,7 +1873,11 @@
           <t>mute</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>mute(1)</t>
+        </is>
+      </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1635,7 +1895,11 @@
           <t>viral</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr"/>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>viral(1)</t>
+        </is>
+      </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1653,7 +1917,11 @@
           <t>filter</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr"/>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>filter(1)</t>
+        </is>
+      </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1671,7 +1939,11 @@
           <t>DM</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr"/>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>DM(1)</t>
+        </is>
+      </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1689,7 +1961,11 @@
           <t>likes, boost</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr"/>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>likes(1), boost(1)</t>
+        </is>
+      </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1707,7 +1983,11 @@
           <t>unfollow</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr"/>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>unfollow(1)</t>
+        </is>
+      </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1725,7 +2005,11 @@
           <t>Q&amp;A</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Q&amp;A(1)</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1743,7 +2027,11 @@
           <t>reach</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>reach(1)</t>
+        </is>
+      </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1761,7 +2049,11 @@
           <t>bio</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr"/>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>bio(1)</t>
+        </is>
+      </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1779,7 +2071,11 @@
           <t>targeted</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr"/>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>targeted(1)</t>
+        </is>
+      </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1797,7 +2093,11 @@
           <t>thread</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr"/>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>thread(1)</t>
+        </is>
+      </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1815,7 +2115,11 @@
           <t>screenshot</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr"/>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>screenshot(1)</t>
+        </is>
+      </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1833,7 +2137,11 @@
           <t>review</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr"/>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>review(2)</t>
+        </is>
+      </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1851,7 +2159,11 @@
           <t>content calendar</t>
         </is>
       </c>
-      <c r="C79" s="3" t="inlineStr"/>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>content(1), calendar(1)</t>
+        </is>
+      </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1869,7 +2181,11 @@
           <t>meme</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr"/>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>meme(1)</t>
+        </is>
+      </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1887,7 +2203,11 @@
           <t>pin</t>
         </is>
       </c>
-      <c r="C81" s="3" t="inlineStr"/>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>pin(1)</t>
+        </is>
+      </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1905,7 +2225,11 @@
           <t>feed</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr"/>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>feed(1)</t>
+        </is>
+      </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1923,7 +2247,11 @@
           <t>engaging</t>
         </is>
       </c>
-      <c r="C83" s="3" t="inlineStr"/>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>engaging(1)</t>
+        </is>
+      </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1941,7 +2269,11 @@
           <t>subscribe, YouTube</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr"/>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>subscribe(1), YouTube(1)</t>
+        </is>
+      </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1959,7 +2291,11 @@
           <t>analytics</t>
         </is>
       </c>
-      <c r="C85" s="3" t="inlineStr"/>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>analytics(1)</t>
+        </is>
+      </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1977,7 +2313,11 @@
           <t>collab</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr"/>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>collab(2)</t>
+        </is>
+      </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -1995,7 +2335,11 @@
           <t>email</t>
         </is>
       </c>
-      <c r="C87" s="3" t="inlineStr"/>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>email(1)</t>
+        </is>
+      </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2013,7 +2357,11 @@
           <t>meeting</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr"/>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>meeting(1)</t>
+        </is>
+      </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2031,7 +2379,11 @@
           <t>presentation</t>
         </is>
       </c>
-      <c r="C89" s="3" t="inlineStr"/>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>presentation(1)</t>
+        </is>
+      </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2049,7 +2401,11 @@
           <t>deadline</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr"/>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>deadline(1)</t>
+        </is>
+      </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2067,7 +2423,11 @@
           <t>Teams</t>
         </is>
       </c>
-      <c r="C91" s="3" t="inlineStr"/>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Teams(1)</t>
+        </is>
+      </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2085,7 +2445,11 @@
           <t>follow up</t>
         </is>
       </c>
-      <c r="C92" s="3" t="inlineStr"/>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>follow(2), up(1)</t>
+        </is>
+      </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2103,7 +2467,11 @@
           <t>report</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr"/>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>report(1)</t>
+        </is>
+      </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2121,7 +2489,11 @@
           <t>schedule</t>
         </is>
       </c>
-      <c r="C94" s="3" t="inlineStr"/>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>schedule(1)</t>
+        </is>
+      </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2139,7 +2511,11 @@
           <t>update</t>
         </is>
       </c>
-      <c r="C95" s="3" t="inlineStr"/>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>update(2)</t>
+        </is>
+      </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2157,7 +2533,11 @@
           <t>CC</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr"/>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>CC(1)</t>
+        </is>
+      </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2175,7 +2555,11 @@
           <t>conference call</t>
         </is>
       </c>
-      <c r="C97" s="3" t="inlineStr"/>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>conference(1), call(1)</t>
+        </is>
+      </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2193,7 +2577,11 @@
           <t>agenda</t>
         </is>
       </c>
-      <c r="C98" s="3" t="inlineStr"/>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>agenda(1)</t>
+        </is>
+      </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2211,7 +2599,11 @@
           <t>attach</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr"/>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>attach(1)</t>
+        </is>
+      </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2229,7 +2621,11 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="C100" s="3" t="inlineStr"/>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>draft(1)</t>
+        </is>
+      </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2247,7 +2643,11 @@
           <t>feedback</t>
         </is>
       </c>
-      <c r="C101" s="3" t="inlineStr"/>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>feedback(1)</t>
+        </is>
+      </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2265,7 +2665,11 @@
           <t>Outlook</t>
         </is>
       </c>
-      <c r="C102" s="3" t="inlineStr"/>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Outlook(1)</t>
+        </is>
+      </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2283,7 +2687,11 @@
           <t>Zoom</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr"/>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>Zoom(1)</t>
+        </is>
+      </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2301,7 +2709,11 @@
           <t>Workday</t>
         </is>
       </c>
-      <c r="C104" s="3" t="inlineStr"/>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Workday(1)</t>
+        </is>
+      </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2319,7 +2731,11 @@
           <t>reschedule</t>
         </is>
       </c>
-      <c r="C105" s="3" t="inlineStr"/>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>reschedule(1)</t>
+        </is>
+      </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2337,7 +2753,11 @@
           <t>aligned</t>
         </is>
       </c>
-      <c r="C106" s="3" t="inlineStr"/>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>aligned(1)</t>
+        </is>
+      </c>
       <c r="D106" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2355,7 +2775,11 @@
           <t>recap</t>
         </is>
       </c>
-      <c r="C107" s="3" t="inlineStr"/>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>recap(1)</t>
+        </is>
+      </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2373,7 +2797,11 @@
           <t>kickoff meeting</t>
         </is>
       </c>
-      <c r="C108" s="3" t="inlineStr"/>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>kickoff(1), meeting(2)</t>
+        </is>
+      </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2391,7 +2819,11 @@
           <t>approve</t>
         </is>
       </c>
-      <c r="C109" s="3" t="inlineStr"/>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>approve(1)</t>
+        </is>
+      </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2409,7 +2841,11 @@
           <t>onboarding</t>
         </is>
       </c>
-      <c r="C110" s="3" t="inlineStr"/>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>onboarding(1)</t>
+        </is>
+      </c>
       <c r="D110" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2427,7 +2863,11 @@
           <t>SharePoint</t>
         </is>
       </c>
-      <c r="C111" s="3" t="inlineStr"/>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>SharePoint(1)</t>
+        </is>
+      </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2445,7 +2885,11 @@
           <t>roadmap</t>
         </is>
       </c>
-      <c r="C112" s="3" t="inlineStr"/>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>roadmap(1)</t>
+        </is>
+      </c>
       <c r="D112" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2463,7 +2907,11 @@
           <t>document</t>
         </is>
       </c>
-      <c r="C113" s="3" t="inlineStr"/>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>document(1)</t>
+        </is>
+      </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2481,7 +2929,11 @@
           <t>performance review</t>
         </is>
       </c>
-      <c r="C114" s="3" t="inlineStr"/>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>performance(1), review(3)</t>
+        </is>
+      </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2499,7 +2951,11 @@
           <t>minutes</t>
         </is>
       </c>
-      <c r="C115" s="3" t="inlineStr"/>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>minutes(1)</t>
+        </is>
+      </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2517,7 +2973,11 @@
           <t>budget</t>
         </is>
       </c>
-      <c r="C116" s="3" t="inlineStr"/>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>budget(1)</t>
+        </is>
+      </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2535,7 +2995,11 @@
           <t>hybrid</t>
         </is>
       </c>
-      <c r="C117" s="3" t="inlineStr"/>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>hybrid(1)</t>
+        </is>
+      </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2553,7 +3017,11 @@
           <t>invoice</t>
         </is>
       </c>
-      <c r="C118" s="3" t="inlineStr"/>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>invoice(1)</t>
+        </is>
+      </c>
       <c r="D118" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2571,7 +3039,11 @@
           <t>stakeholder alignment</t>
         </is>
       </c>
-      <c r="C119" s="3" t="inlineStr"/>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>stakeholder(1), alignment(1)</t>
+        </is>
+      </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2589,7 +3061,11 @@
           <t>workflow</t>
         </is>
       </c>
-      <c r="C120" s="3" t="inlineStr"/>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>workflow(1)</t>
+        </is>
+      </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2607,7 +3083,11 @@
           <t>slides</t>
         </is>
       </c>
-      <c r="C121" s="3" t="inlineStr"/>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>slides(1)</t>
+        </is>
+      </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2625,7 +3105,11 @@
           <t>virtual</t>
         </is>
       </c>
-      <c r="C122" s="3" t="inlineStr"/>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>virtual(1)</t>
+        </is>
+      </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2643,7 +3127,11 @@
           <t>sync</t>
         </is>
       </c>
-      <c r="C123" s="3" t="inlineStr"/>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>sync(1)</t>
+        </is>
+      </c>
       <c r="D123" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2661,7 +3149,11 @@
           <t>OKR</t>
         </is>
       </c>
-      <c r="C124" s="3" t="inlineStr"/>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>OKR(1)</t>
+        </is>
+      </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2679,7 +3171,11 @@
           <t>reminder</t>
         </is>
       </c>
-      <c r="C125" s="3" t="inlineStr"/>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>reminder(1)</t>
+        </is>
+      </c>
       <c r="D125" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2697,7 +3193,11 @@
           <t>town hall</t>
         </is>
       </c>
-      <c r="C126" s="3" t="inlineStr"/>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>town(1), hall(1)</t>
+        </is>
+      </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2715,7 +3215,11 @@
           <t>battery</t>
         </is>
       </c>
-      <c r="C127" s="3" t="inlineStr"/>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>battery(1)</t>
+        </is>
+      </c>
       <c r="D127" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2733,7 +3237,11 @@
           <t>WiFi</t>
         </is>
       </c>
-      <c r="C128" s="3" t="inlineStr"/>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>WiFi(2)</t>
+        </is>
+      </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2751,7 +3259,11 @@
           <t>app</t>
         </is>
       </c>
-      <c r="C129" s="3" t="inlineStr"/>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>app(1)</t>
+        </is>
+      </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2769,7 +3281,11 @@
           <t>restart</t>
         </is>
       </c>
-      <c r="C130" s="3" t="inlineStr"/>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>restart(1)</t>
+        </is>
+      </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2787,7 +3303,11 @@
           <t>update</t>
         </is>
       </c>
-      <c r="C131" s="3" t="inlineStr"/>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>update(3)</t>
+        </is>
+      </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2805,7 +3325,11 @@
           <t>reset</t>
         </is>
       </c>
-      <c r="C132" s="3" t="inlineStr"/>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>reset(1)</t>
+        </is>
+      </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2823,7 +3347,11 @@
           <t>Bluetooth</t>
         </is>
       </c>
-      <c r="C133" s="3" t="inlineStr"/>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Bluetooth(2)</t>
+        </is>
+      </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2841,7 +3369,11 @@
           <t>notification</t>
         </is>
       </c>
-      <c r="C134" s="3" t="inlineStr"/>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>notification(1)</t>
+        </is>
+      </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2859,7 +3391,11 @@
           <t>backup</t>
         </is>
       </c>
-      <c r="C135" s="3" t="inlineStr"/>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>backup(2)</t>
+        </is>
+      </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2877,7 +3413,11 @@
           <t>software</t>
         </is>
       </c>
-      <c r="C136" s="3" t="inlineStr"/>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>software(1)</t>
+        </is>
+      </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2895,7 +3435,11 @@
           <t>cloud</t>
         </is>
       </c>
-      <c r="C137" s="3" t="inlineStr"/>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>cloud(2)</t>
+        </is>
+      </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2913,7 +3457,11 @@
           <t>USB</t>
         </is>
       </c>
-      <c r="C138" s="3" t="inlineStr"/>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>USB(2)</t>
+        </is>
+      </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2931,7 +3479,11 @@
           <t>factory reset</t>
         </is>
       </c>
-      <c r="C139" s="3" t="inlineStr"/>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>factory(1), reset(2)</t>
+        </is>
+      </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2949,7 +3501,11 @@
           <t>charger</t>
         </is>
       </c>
-      <c r="C140" s="3" t="inlineStr"/>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>charger(1)</t>
+        </is>
+      </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2967,7 +3523,11 @@
           <t>dark mode</t>
         </is>
       </c>
-      <c r="C141" s="3" t="inlineStr"/>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>dark(1), mode(1)</t>
+        </is>
+      </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -2985,7 +3545,11 @@
           <t>screen protector</t>
         </is>
       </c>
-      <c r="C142" s="3" t="inlineStr"/>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>screen(1), protector(1)</t>
+        </is>
+      </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3003,7 +3567,11 @@
           <t>pair</t>
         </is>
       </c>
-      <c r="C143" s="3" t="inlineStr"/>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>pair(1)</t>
+        </is>
+      </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3021,7 +3589,11 @@
           <t>cache</t>
         </is>
       </c>
-      <c r="C144" s="3" t="inlineStr"/>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>cache(1)</t>
+        </is>
+      </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3039,7 +3611,11 @@
           <t>hard reset</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr"/>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>hard(1), reset(3)</t>
+        </is>
+      </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3057,7 +3633,11 @@
           <t>WiFi</t>
         </is>
       </c>
-      <c r="C146" s="3" t="inlineStr"/>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>WiFi(3)</t>
+        </is>
+      </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3075,7 +3655,11 @@
           <t>storage</t>
         </is>
       </c>
-      <c r="C147" s="3" t="inlineStr"/>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>storage(1)</t>
+        </is>
+      </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3093,7 +3677,11 @@
           <t>charging</t>
         </is>
       </c>
-      <c r="C148" s="3" t="inlineStr"/>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>charging(1)</t>
+        </is>
+      </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3111,7 +3699,11 @@
           <t>sync</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr"/>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>sync(2)</t>
+        </is>
+      </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3129,7 +3721,11 @@
           <t>fingerprint</t>
         </is>
       </c>
-      <c r="C150" s="3" t="inlineStr"/>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>fingerprint(1)</t>
+        </is>
+      </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3147,7 +3743,11 @@
           <t>reboot</t>
         </is>
       </c>
-      <c r="C151" s="3" t="inlineStr"/>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>reboot(1)</t>
+        </is>
+      </c>
       <c r="D151" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3165,7 +3765,11 @@
           <t>signal</t>
         </is>
       </c>
-      <c r="C152" s="3" t="inlineStr"/>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>signal(1)</t>
+        </is>
+      </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3183,7 +3787,11 @@
           <t>firmware</t>
         </is>
       </c>
-      <c r="C153" s="3" t="inlineStr"/>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>firmware(1)</t>
+        </is>
+      </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3201,7 +3809,11 @@
           <t>speaker</t>
         </is>
       </c>
-      <c r="C154" s="3" t="inlineStr"/>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>speaker(2)</t>
+        </is>
+      </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3219,7 +3831,11 @@
           <t>calibration</t>
         </is>
       </c>
-      <c r="C155" s="3" t="inlineStr"/>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>calibration(1)</t>
+        </is>
+      </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3237,7 +3853,11 @@
           <t>fast charging</t>
         </is>
       </c>
-      <c r="C156" s="3" t="inlineStr"/>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>fast(1), charging(2)</t>
+        </is>
+      </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3255,7 +3875,11 @@
           <t>microphone</t>
         </is>
       </c>
-      <c r="C157" s="3" t="inlineStr"/>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>microphone(1)</t>
+        </is>
+      </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3273,7 +3897,11 @@
           <t>format</t>
         </is>
       </c>
-      <c r="C158" s="3" t="inlineStr"/>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>format(1)</t>
+        </is>
+      </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3291,7 +3919,11 @@
           <t>rollback</t>
         </is>
       </c>
-      <c r="C159" s="3" t="inlineStr"/>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>rollback(1)</t>
+        </is>
+      </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3309,7 +3941,11 @@
           <t>notification</t>
         </is>
       </c>
-      <c r="C160" s="3" t="inlineStr"/>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>notification(2)</t>
+        </is>
+      </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3327,7 +3963,11 @@
           <t>GPS</t>
         </is>
       </c>
-      <c r="C161" s="3" t="inlineStr"/>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>GPS(1)</t>
+        </is>
+      </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3345,7 +3985,11 @@
           <t>lag</t>
         </is>
       </c>
-      <c r="C162" s="3" t="inlineStr"/>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>lag(1)</t>
+        </is>
+      </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3363,7 +4007,11 @@
           <t>disable</t>
         </is>
       </c>
-      <c r="C163" s="3" t="inlineStr"/>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>disable(1)</t>
+        </is>
+      </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3381,7 +4029,11 @@
           <t>driver</t>
         </is>
       </c>
-      <c r="C164" s="3" t="inlineStr"/>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>driver(1)</t>
+        </is>
+      </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3399,7 +4051,11 @@
           <t>uninstall</t>
         </is>
       </c>
-      <c r="C165" s="3" t="inlineStr"/>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>uninstall(1)</t>
+        </is>
+      </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3417,7 +4073,11 @@
           <t>resolution</t>
         </is>
       </c>
-      <c r="C166" s="3" t="inlineStr"/>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>resolution(1)</t>
+        </is>
+      </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3435,7 +4095,11 @@
           <t>Uber</t>
         </is>
       </c>
-      <c r="C167" s="3" t="inlineStr"/>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Uber(1)</t>
+        </is>
+      </c>
       <c r="D167" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3453,7 +4117,11 @@
           <t>Starbucks</t>
         </is>
       </c>
-      <c r="C168" s="3" t="inlineStr"/>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Starbucks(1)</t>
+        </is>
+      </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3471,7 +4139,11 @@
           <t>Netflix</t>
         </is>
       </c>
-      <c r="C169" s="3" t="inlineStr"/>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>Netflix(1)</t>
+        </is>
+      </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3489,7 +4161,11 @@
           <t>Spotify</t>
         </is>
       </c>
-      <c r="C170" s="3" t="inlineStr"/>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>Spotify(1)</t>
+        </is>
+      </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3507,7 +4183,11 @@
           <t>Apple Pay</t>
         </is>
       </c>
-      <c r="C171" s="3" t="inlineStr"/>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Apple(1), Pay(1)</t>
+        </is>
+      </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3525,7 +4205,11 @@
           <t>wallet</t>
         </is>
       </c>
-      <c r="C172" s="3" t="inlineStr"/>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>wallet(1)</t>
+        </is>
+      </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3543,7 +4227,11 @@
           <t>HungerStation</t>
         </is>
       </c>
-      <c r="C173" s="3" t="inlineStr"/>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>HungerStation(1)</t>
+        </is>
+      </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3561,7 +4249,11 @@
           <t>Netflix</t>
         </is>
       </c>
-      <c r="C174" s="3" t="inlineStr"/>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>Netflix(2)</t>
+        </is>
+      </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3579,7 +4271,11 @@
           <t>discount</t>
         </is>
       </c>
-      <c r="C175" s="3" t="inlineStr"/>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>discount(1)</t>
+        </is>
+      </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3597,7 +4293,11 @@
           <t>Almosafer</t>
         </is>
       </c>
-      <c r="C176" s="3" t="inlineStr"/>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>Almosafer(1)</t>
+        </is>
+      </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3615,7 +4315,11 @@
           <t>STC Pay</t>
         </is>
       </c>
-      <c r="C177" s="3" t="inlineStr"/>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>STC(1), Pay(2)</t>
+        </is>
+      </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3633,7 +4337,11 @@
           <t>delivery</t>
         </is>
       </c>
-      <c r="C178" s="3" t="inlineStr"/>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>delivery(1)</t>
+        </is>
+      </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3651,7 +4359,11 @@
           <t>Careem</t>
         </is>
       </c>
-      <c r="C179" s="3" t="inlineStr"/>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>Careem(1)</t>
+        </is>
+      </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3669,7 +4381,11 @@
           <t>gym</t>
         </is>
       </c>
-      <c r="C180" s="3" t="inlineStr"/>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>gym(1)</t>
+        </is>
+      </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3687,7 +4403,11 @@
           <t>subscription</t>
         </is>
       </c>
-      <c r="C181" s="3" t="inlineStr"/>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>subscription(1)</t>
+        </is>
+      </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3705,7 +4425,11 @@
           <t>fusion food</t>
         </is>
       </c>
-      <c r="C182" s="3" t="inlineStr"/>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>fusion(1), food(1)</t>
+        </is>
+      </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3723,7 +4447,11 @@
           <t>appointment</t>
         </is>
       </c>
-      <c r="C183" s="3" t="inlineStr"/>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>appointment(1)</t>
+        </is>
+      </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3741,7 +4469,11 @@
           <t>checkout</t>
         </is>
       </c>
-      <c r="C184" s="3" t="inlineStr"/>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>checkout(1)</t>
+        </is>
+      </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3759,7 +4491,11 @@
           <t>gift card</t>
         </is>
       </c>
-      <c r="C185" s="3" t="inlineStr"/>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>gift(1), card(1)</t>
+        </is>
+      </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3777,7 +4513,11 @@
           <t>full board</t>
         </is>
       </c>
-      <c r="C186" s="3" t="inlineStr"/>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>full(1), board(1)</t>
+        </is>
+      </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3795,7 +4535,11 @@
           <t>loyalty points</t>
         </is>
       </c>
-      <c r="C187" s="3" t="inlineStr"/>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>loyalty(1), points(1)</t>
+        </is>
+      </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3813,7 +4557,11 @@
           <t>meditation</t>
         </is>
       </c>
-      <c r="C188" s="3" t="inlineStr"/>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>meditation(1)</t>
+        </is>
+      </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3831,7 +4579,11 @@
           <t>oat milk</t>
         </is>
       </c>
-      <c r="C189" s="3" t="inlineStr"/>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>oat(1), milk(1)</t>
+        </is>
+      </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3849,7 +4601,11 @@
           <t>happy hour</t>
         </is>
       </c>
-      <c r="C190" s="3" t="inlineStr"/>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>happy(1), hour(1)</t>
+        </is>
+      </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3867,7 +4623,11 @@
           <t>premium</t>
         </is>
       </c>
-      <c r="C191" s="3" t="inlineStr"/>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>premium(1)</t>
+        </is>
+      </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3885,7 +4645,11 @@
           <t>reservation</t>
         </is>
       </c>
-      <c r="C192" s="3" t="inlineStr"/>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>reservation(1)</t>
+        </is>
+      </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3903,7 +4667,11 @@
           <t>economy</t>
         </is>
       </c>
-      <c r="C193" s="3" t="inlineStr"/>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>economy(1)</t>
+        </is>
+      </c>
       <c r="D193" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3921,7 +4689,11 @@
           <t>cashback</t>
         </is>
       </c>
-      <c r="C194" s="3" t="inlineStr"/>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>cashback(1)</t>
+        </is>
+      </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3939,7 +4711,11 @@
           <t>membership</t>
         </is>
       </c>
-      <c r="C195" s="3" t="inlineStr"/>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>membership(1)</t>
+        </is>
+      </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3957,7 +4733,11 @@
           <t>brunch</t>
         </is>
       </c>
-      <c r="C196" s="3" t="inlineStr"/>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>brunch(1)</t>
+        </is>
+      </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3975,7 +4755,11 @@
           <t>concert</t>
         </is>
       </c>
-      <c r="C197" s="3" t="inlineStr"/>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>concert(1)</t>
+        </is>
+      </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -3993,7 +4777,11 @@
           <t>spa</t>
         </is>
       </c>
-      <c r="C198" s="3" t="inlineStr"/>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>spa(1)</t>
+        </is>
+      </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4011,7 +4799,11 @@
           <t>trial</t>
         </is>
       </c>
-      <c r="C199" s="3" t="inlineStr"/>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>trial(1)</t>
+        </is>
+      </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4029,7 +4821,11 @@
           <t>streaming</t>
         </is>
       </c>
-      <c r="C200" s="3" t="inlineStr"/>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>streaming(1)</t>
+        </is>
+      </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4047,7 +4843,11 @@
           <t>takeaway</t>
         </is>
       </c>
-      <c r="C201" s="3" t="inlineStr"/>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>takeaway(1)</t>
+        </is>
+      </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4065,7 +4865,11 @@
           <t>layover</t>
         </is>
       </c>
-      <c r="C202" s="3" t="inlineStr"/>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>layover(1)</t>
+        </is>
+      </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4083,7 +4887,11 @@
           <t>massage</t>
         </is>
       </c>
-      <c r="C203" s="3" t="inlineStr"/>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>massage(1)</t>
+        </is>
+      </c>
       <c r="D203" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4101,7 +4909,11 @@
           <t>promo code</t>
         </is>
       </c>
-      <c r="C204" s="3" t="inlineStr"/>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>promo(1), code(2)</t>
+        </is>
+      </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4119,7 +4931,11 @@
           <t>specialty</t>
         </is>
       </c>
-      <c r="C205" s="3" t="inlineStr"/>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>specialty(1)</t>
+        </is>
+      </c>
       <c r="D205" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4137,7 +4953,11 @@
           <t>check-in</t>
         </is>
       </c>
-      <c r="C206" s="3" t="inlineStr"/>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>check-in(1)</t>
+        </is>
+      </c>
       <c r="D206" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4155,7 +4975,11 @@
           <t>voucher</t>
         </is>
       </c>
-      <c r="C207" s="3" t="inlineStr"/>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>voucher(1)</t>
+        </is>
+      </c>
       <c r="D207" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4173,7 +4997,11 @@
           <t>gift</t>
         </is>
       </c>
-      <c r="C208" s="3" t="inlineStr"/>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>gift(2)</t>
+        </is>
+      </c>
       <c r="D208" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4191,7 +5019,11 @@
           <t>reward points</t>
         </is>
       </c>
-      <c r="C209" s="3" t="inlineStr"/>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>reward(1), points(2)</t>
+        </is>
+      </c>
       <c r="D209" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4209,7 +5041,11 @@
           <t>daily deals</t>
         </is>
       </c>
-      <c r="C210" s="3" t="inlineStr"/>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>daily(1), deals(1)</t>
+        </is>
+      </c>
       <c r="D210" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4227,7 +5063,11 @@
           <t>delivery</t>
         </is>
       </c>
-      <c r="C211" s="3" t="inlineStr"/>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>delivery(2)</t>
+        </is>
+      </c>
       <c r="D211" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4245,7 +5085,11 @@
           <t>cart</t>
         </is>
       </c>
-      <c r="C212" s="3" t="inlineStr"/>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>cart(1)</t>
+        </is>
+      </c>
       <c r="D212" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4263,7 +5107,11 @@
           <t>checkout</t>
         </is>
       </c>
-      <c r="C213" s="3" t="inlineStr"/>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>checkout(2)</t>
+        </is>
+      </c>
       <c r="D213" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4281,7 +5129,11 @@
           <t>coupon</t>
         </is>
       </c>
-      <c r="C214" s="3" t="inlineStr"/>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>coupon(1)</t>
+        </is>
+      </c>
       <c r="D214" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4299,7 +5151,11 @@
           <t>sale</t>
         </is>
       </c>
-      <c r="C215" s="3" t="inlineStr"/>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>sale(1)</t>
+        </is>
+      </c>
       <c r="D215" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4317,7 +5173,11 @@
           <t>shipping</t>
         </is>
       </c>
-      <c r="C216" s="3" t="inlineStr"/>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>shipping(1)</t>
+        </is>
+      </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4335,7 +5195,11 @@
           <t>review</t>
         </is>
       </c>
-      <c r="C217" s="3" t="inlineStr"/>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>review(4)</t>
+        </is>
+      </c>
       <c r="D217" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4353,7 +5217,11 @@
           <t>rating</t>
         </is>
       </c>
-      <c r="C218" s="3" t="inlineStr"/>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>rating(1)</t>
+        </is>
+      </c>
       <c r="D218" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4371,7 +5239,11 @@
           <t>return</t>
         </is>
       </c>
-      <c r="C219" s="3" t="inlineStr"/>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>return(1)</t>
+        </is>
+      </c>
       <c r="D219" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4389,7 +5261,11 @@
           <t>promo code</t>
         </is>
       </c>
-      <c r="C220" s="3" t="inlineStr"/>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>promo(2), code(3)</t>
+        </is>
+      </c>
       <c r="D220" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4407,7 +5283,11 @@
           <t>order</t>
         </is>
       </c>
-      <c r="C221" s="3" t="inlineStr"/>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>order(1)</t>
+        </is>
+      </c>
       <c r="D221" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4425,7 +5305,11 @@
           <t>stock</t>
         </is>
       </c>
-      <c r="C222" s="3" t="inlineStr"/>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>stock(1)</t>
+        </is>
+      </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4443,7 +5327,11 @@
           <t>Noon</t>
         </is>
       </c>
-      <c r="C223" s="3" t="inlineStr"/>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>Noon(1)</t>
+        </is>
+      </c>
       <c r="D223" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4461,7 +5349,11 @@
           <t>compare</t>
         </is>
       </c>
-      <c r="C224" s="3" t="inlineStr"/>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>compare(1)</t>
+        </is>
+      </c>
       <c r="D224" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4479,7 +5371,11 @@
           <t>delivery</t>
         </is>
       </c>
-      <c r="C225" s="3" t="inlineStr"/>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>delivery(3)</t>
+        </is>
+      </c>
       <c r="D225" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4497,7 +5393,11 @@
           <t>wishlist</t>
         </is>
       </c>
-      <c r="C226" s="3" t="inlineStr"/>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>wishlist(1)</t>
+        </is>
+      </c>
       <c r="D226" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4515,7 +5415,11 @@
           <t>chat</t>
         </is>
       </c>
-      <c r="C227" s="3" t="inlineStr"/>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>chat(1)</t>
+        </is>
+      </c>
       <c r="D227" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4533,7 +5437,11 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C228" s="3" t="inlineStr"/>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>Amazon(1)</t>
+        </is>
+      </c>
       <c r="D228" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4551,7 +5459,11 @@
           <t>damaged</t>
         </is>
       </c>
-      <c r="C229" s="3" t="inlineStr"/>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>damaged(1)</t>
+        </is>
+      </c>
       <c r="D229" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4569,7 +5481,11 @@
           <t>filter</t>
         </is>
       </c>
-      <c r="C230" s="3" t="inlineStr"/>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>filter(2)</t>
+        </is>
+      </c>
       <c r="D230" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4587,7 +5503,11 @@
           <t>refund</t>
         </is>
       </c>
-      <c r="C231" s="3" t="inlineStr"/>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>refund(1)</t>
+        </is>
+      </c>
       <c r="D231" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4605,7 +5525,11 @@
           <t>cashback</t>
         </is>
       </c>
-      <c r="C232" s="3" t="inlineStr"/>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>cashback(2)</t>
+        </is>
+      </c>
       <c r="D232" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4623,7 +5547,11 @@
           <t>tracking number</t>
         </is>
       </c>
-      <c r="C233" s="3" t="inlineStr"/>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>tracking(1), number(1)</t>
+        </is>
+      </c>
       <c r="D233" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4641,7 +5569,11 @@
           <t>Shein</t>
         </is>
       </c>
-      <c r="C234" s="3" t="inlineStr"/>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>Shein(1)</t>
+        </is>
+      </c>
       <c r="D234" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4659,7 +5591,11 @@
           <t>subscribe</t>
         </is>
       </c>
-      <c r="C235" s="3" t="inlineStr"/>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>subscribe(2)</t>
+        </is>
+      </c>
       <c r="D235" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4677,7 +5613,11 @@
           <t>warranty</t>
         </is>
       </c>
-      <c r="C236" s="3" t="inlineStr"/>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>warranty(1)</t>
+        </is>
+      </c>
       <c r="D236" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4695,7 +5635,11 @@
           <t>installment</t>
         </is>
       </c>
-      <c r="C237" s="3" t="inlineStr"/>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>installment(1)</t>
+        </is>
+      </c>
       <c r="D237" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4713,7 +5657,11 @@
           <t>compare</t>
         </is>
       </c>
-      <c r="C238" s="3" t="inlineStr"/>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>compare(2)</t>
+        </is>
+      </c>
       <c r="D238" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4731,7 +5679,11 @@
           <t>flash sale</t>
         </is>
       </c>
-      <c r="C239" s="3" t="inlineStr"/>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>flash(1), sale(2)</t>
+        </is>
+      </c>
       <c r="D239" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4749,7 +5701,11 @@
           <t>payment method</t>
         </is>
       </c>
-      <c r="C240" s="3" t="inlineStr"/>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>payment(1), method(1)</t>
+        </is>
+      </c>
       <c r="D240" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4767,7 +5723,11 @@
           <t>confirmed</t>
         </is>
       </c>
-      <c r="C241" s="3" t="inlineStr"/>
+      <c r="C241" s="3" t="inlineStr">
+        <is>
+          <t>confirmed(1)</t>
+        </is>
+      </c>
       <c r="D241" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4785,7 +5745,11 @@
           <t>free shipping</t>
         </is>
       </c>
-      <c r="C242" s="3" t="inlineStr"/>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>free(1), shipping(2)</t>
+        </is>
+      </c>
       <c r="D242" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4803,7 +5767,11 @@
           <t>return</t>
         </is>
       </c>
-      <c r="C243" s="3" t="inlineStr"/>
+      <c r="C243" s="3" t="inlineStr">
+        <is>
+          <t>return(2)</t>
+        </is>
+      </c>
       <c r="D243" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4821,7 +5789,11 @@
           <t>invoice</t>
         </is>
       </c>
-      <c r="C244" s="3" t="inlineStr"/>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>invoice(2)</t>
+        </is>
+      </c>
       <c r="D244" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4839,7 +5811,11 @@
           <t>bug</t>
         </is>
       </c>
-      <c r="C245" s="3" t="inlineStr"/>
+      <c r="C245" s="3" t="inlineStr">
+        <is>
+          <t>bug(2)</t>
+        </is>
+      </c>
       <c r="D245" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4857,7 +5833,11 @@
           <t>Jarir, order</t>
         </is>
       </c>
-      <c r="C246" s="3" t="inlineStr"/>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>Jarir(1), order(2)</t>
+        </is>
+      </c>
       <c r="D246" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4875,7 +5855,11 @@
           <t>checkout</t>
         </is>
       </c>
-      <c r="C247" s="3" t="inlineStr"/>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>checkout(3)</t>
+        </is>
+      </c>
       <c r="D247" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4893,7 +5877,11 @@
           <t>variant</t>
         </is>
       </c>
-      <c r="C248" s="3" t="inlineStr"/>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>variant(1)</t>
+        </is>
+      </c>
       <c r="D248" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4911,7 +5899,11 @@
           <t>voucher</t>
         </is>
       </c>
-      <c r="C249" s="3" t="inlineStr"/>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>voucher(2)</t>
+        </is>
+      </c>
       <c r="D249" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4929,7 +5921,11 @@
           <t>detailed</t>
         </is>
       </c>
-      <c r="C250" s="3" t="inlineStr"/>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>detailed(1)</t>
+        </is>
+      </c>
       <c r="D250" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4947,7 +5943,11 @@
           <t>slot</t>
         </is>
       </c>
-      <c r="C251" s="3" t="inlineStr"/>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>slot(1)</t>
+        </is>
+      </c>
       <c r="D251" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4965,7 +5965,11 @@
           <t>loyalty program</t>
         </is>
       </c>
-      <c r="C252" s="3" t="inlineStr"/>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>loyalty(2), program(1)</t>
+        </is>
+      </c>
       <c r="D252" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -4983,7 +5987,11 @@
           <t>discount code</t>
         </is>
       </c>
-      <c r="C253" s="3" t="inlineStr"/>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>discount(2), code(4)</t>
+        </is>
+      </c>
       <c r="D253" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5001,7 +6009,11 @@
           <t>payment</t>
         </is>
       </c>
-      <c r="C254" s="3" t="inlineStr"/>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>payment(2)</t>
+        </is>
+      </c>
       <c r="D254" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5019,7 +6031,11 @@
           <t>exchange</t>
         </is>
       </c>
-      <c r="C255" s="3" t="inlineStr"/>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>exchange(1)</t>
+        </is>
+      </c>
       <c r="D255" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5037,7 +6053,11 @@
           <t>browse</t>
         </is>
       </c>
-      <c r="C256" s="3" t="inlineStr"/>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>browse(1)</t>
+        </is>
+      </c>
       <c r="D256" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5055,7 +6075,11 @@
           <t>WhatsApp</t>
         </is>
       </c>
-      <c r="C257" s="3" t="inlineStr"/>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp(1)</t>
+        </is>
+      </c>
       <c r="D257" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5073,7 +6097,11 @@
           <t>SMS</t>
         </is>
       </c>
-      <c r="C258" s="3" t="inlineStr"/>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>SMS(1)</t>
+        </is>
+      </c>
       <c r="D258" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5091,7 +6119,11 @@
           <t>screenshot</t>
         </is>
       </c>
-      <c r="C259" s="3" t="inlineStr"/>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>screenshot(2)</t>
+        </is>
+      </c>
       <c r="D259" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5109,7 +6141,11 @@
           <t>Play Store</t>
         </is>
       </c>
-      <c r="C260" s="3" t="inlineStr"/>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>Play(1), Store(2)</t>
+        </is>
+      </c>
       <c r="D260" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5127,7 +6163,11 @@
           <t>install</t>
         </is>
       </c>
-      <c r="C261" s="3" t="inlineStr"/>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>install(1)</t>
+        </is>
+      </c>
       <c r="D261" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5145,7 +6185,11 @@
           <t>uninstall</t>
         </is>
       </c>
-      <c r="C262" s="3" t="inlineStr"/>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>uninstall(2)</t>
+        </is>
+      </c>
       <c r="D262" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5163,7 +6207,11 @@
           <t>notification</t>
         </is>
       </c>
-      <c r="C263" s="3" t="inlineStr"/>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>notification(3)</t>
+        </is>
+      </c>
       <c r="D263" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5181,7 +6229,11 @@
           <t>update</t>
         </is>
       </c>
-      <c r="C264" s="3" t="inlineStr"/>
+      <c r="C264" s="3" t="inlineStr">
+        <is>
+          <t>update(4)</t>
+        </is>
+      </c>
       <c r="D264" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5199,7 +6251,11 @@
           <t>Bluetooth</t>
         </is>
       </c>
-      <c r="C265" s="3" t="inlineStr"/>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>Bluetooth(3)</t>
+        </is>
+      </c>
       <c r="D265" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5217,7 +6273,11 @@
           <t>contacts</t>
         </is>
       </c>
-      <c r="C266" s="3" t="inlineStr"/>
+      <c r="C266" s="3" t="inlineStr">
+        <is>
+          <t>contacts(1)</t>
+        </is>
+      </c>
       <c r="D266" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5235,7 +6295,11 @@
           <t>backup, cloud</t>
         </is>
       </c>
-      <c r="C267" s="3" t="inlineStr"/>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>backup(3), cloud(3)</t>
+        </is>
+      </c>
       <c r="D267" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5253,7 +6317,11 @@
           <t>notification</t>
         </is>
       </c>
-      <c r="C268" s="3" t="inlineStr"/>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>notification(4)</t>
+        </is>
+      </c>
       <c r="D268" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5271,7 +6339,11 @@
           <t>mute</t>
         </is>
       </c>
-      <c r="C269" s="3" t="inlineStr"/>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>mute(2)</t>
+        </is>
+      </c>
       <c r="D269" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5289,7 +6361,11 @@
           <t>voice note</t>
         </is>
       </c>
-      <c r="C270" s="3" t="inlineStr"/>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>voice(1), note(1)</t>
+        </is>
+      </c>
       <c r="D270" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5307,7 +6383,11 @@
           <t>storage</t>
         </is>
       </c>
-      <c r="C271" s="3" t="inlineStr"/>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>storage(2)</t>
+        </is>
+      </c>
       <c r="D271" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5325,7 +6405,11 @@
           <t>forward</t>
         </is>
       </c>
-      <c r="C272" s="3" t="inlineStr"/>
+      <c r="C272" s="3" t="inlineStr">
+        <is>
+          <t>forward(1)</t>
+        </is>
+      </c>
       <c r="D272" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5343,7 +6427,11 @@
           <t>dual SIM</t>
         </is>
       </c>
-      <c r="C273" s="3" t="inlineStr"/>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>dual(1), SIM(1)</t>
+        </is>
+      </c>
       <c r="D273" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5361,7 +6449,11 @@
           <t>restore</t>
         </is>
       </c>
-      <c r="C274" s="3" t="inlineStr"/>
+      <c r="C274" s="3" t="inlineStr">
+        <is>
+          <t>restore(1)</t>
+        </is>
+      </c>
       <c r="D274" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5379,7 +6471,11 @@
           <t>iOS</t>
         </is>
       </c>
-      <c r="C275" s="3" t="inlineStr"/>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>iOS(1)</t>
+        </is>
+      </c>
       <c r="D275" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5397,7 +6493,11 @@
           <t>Careem</t>
         </is>
       </c>
-      <c r="C276" s="3" t="inlineStr"/>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Careem(2)</t>
+        </is>
+      </c>
       <c r="D276" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5415,7 +6515,11 @@
           <t>sync</t>
         </is>
       </c>
-      <c r="C277" s="3" t="inlineStr"/>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>sync(3)</t>
+        </is>
+      </c>
       <c r="D277" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5433,7 +6537,11 @@
           <t>low battery</t>
         </is>
       </c>
-      <c r="C278" s="3" t="inlineStr"/>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>low(1), battery(2)</t>
+        </is>
+      </c>
       <c r="D278" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5451,7 +6559,11 @@
           <t>pair</t>
         </is>
       </c>
-      <c r="C279" s="3" t="inlineStr"/>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>pair(2)</t>
+        </is>
+      </c>
       <c r="D279" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5469,7 +6581,11 @@
           <t>cache</t>
         </is>
       </c>
-      <c r="C280" s="3" t="inlineStr"/>
+      <c r="C280" s="3" t="inlineStr">
+        <is>
+          <t>cache(2)</t>
+        </is>
+      </c>
       <c r="D280" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5487,7 +6603,11 @@
           <t>location share</t>
         </is>
       </c>
-      <c r="C281" s="3" t="inlineStr"/>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>location(1), share(2)</t>
+        </is>
+      </c>
       <c r="D281" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5505,7 +6625,11 @@
           <t>face ID</t>
         </is>
       </c>
-      <c r="C282" s="3" t="inlineStr"/>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>face(1), ID(1)</t>
+        </is>
+      </c>
       <c r="D282" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5523,7 +6647,11 @@
           <t>block</t>
         </is>
       </c>
-      <c r="C283" s="3" t="inlineStr"/>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>block(2)</t>
+        </is>
+      </c>
       <c r="D283" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5541,7 +6669,11 @@
           <t>Snapchat</t>
         </is>
       </c>
-      <c r="C284" s="3" t="inlineStr"/>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>Snapchat(2)</t>
+        </is>
+      </c>
       <c r="D284" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5559,7 +6691,11 @@
           <t>freeze</t>
         </is>
       </c>
-      <c r="C285" s="3" t="inlineStr"/>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>freeze(1)</t>
+        </is>
+      </c>
       <c r="D285" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5577,7 +6713,11 @@
           <t>restart</t>
         </is>
       </c>
-      <c r="C286" s="3" t="inlineStr"/>
+      <c r="C286" s="3" t="inlineStr">
+        <is>
+          <t>restart(2)</t>
+        </is>
+      </c>
       <c r="D286" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5595,7 +6735,11 @@
           <t>signal</t>
         </is>
       </c>
-      <c r="C287" s="3" t="inlineStr"/>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>signal(2)</t>
+        </is>
+      </c>
       <c r="D287" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5613,7 +6757,11 @@
           <t>export</t>
         </is>
       </c>
-      <c r="C288" s="3" t="inlineStr"/>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>export(1)</t>
+        </is>
+      </c>
       <c r="D288" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5631,7 +6779,11 @@
           <t>NFC</t>
         </is>
       </c>
-      <c r="C289" s="3" t="inlineStr"/>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>NFC(1)</t>
+        </is>
+      </c>
       <c r="D289" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5649,7 +6801,11 @@
           <t>verify</t>
         </is>
       </c>
-      <c r="C290" s="3" t="inlineStr"/>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>verify(1)</t>
+        </is>
+      </c>
       <c r="D290" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5667,7 +6823,11 @@
           <t>upload</t>
         </is>
       </c>
-      <c r="C291" s="3" t="inlineStr"/>
+      <c r="C291" s="3" t="inlineStr">
+        <is>
+          <t>upload(1)</t>
+        </is>
+      </c>
       <c r="D291" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5685,7 +6845,11 @@
           <t>permission</t>
         </is>
       </c>
-      <c r="C292" s="3" t="inlineStr"/>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>permission(1)</t>
+        </is>
+      </c>
       <c r="D292" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5703,7 +6867,11 @@
           <t>download</t>
         </is>
       </c>
-      <c r="C293" s="3" t="inlineStr"/>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>download(1)</t>
+        </is>
+      </c>
       <c r="D293" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5721,7 +6889,11 @@
           <t>split screen</t>
         </is>
       </c>
-      <c r="C294" s="3" t="inlineStr"/>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>split(1), screen(2)</t>
+        </is>
+      </c>
       <c r="D294" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5739,7 +6911,11 @@
           <t>report</t>
         </is>
       </c>
-      <c r="C295" s="3" t="inlineStr"/>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>report(2)</t>
+        </is>
+      </c>
       <c r="D295" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5757,7 +6933,11 @@
           <t>update</t>
         </is>
       </c>
-      <c r="C296" s="3" t="inlineStr"/>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>update(5)</t>
+        </is>
+      </c>
       <c r="D296" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5775,7 +6955,11 @@
           <t>hotspot</t>
         </is>
       </c>
-      <c r="C297" s="3" t="inlineStr"/>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>hotspot(1)</t>
+        </is>
+      </c>
       <c r="D297" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5793,7 +6977,11 @@
           <t>wireless charging</t>
         </is>
       </c>
-      <c r="C298" s="3" t="inlineStr"/>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>wireless(1), charging(3)</t>
+        </is>
+      </c>
       <c r="D298" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5811,7 +6999,11 @@
           <t>transfer</t>
         </is>
       </c>
-      <c r="C299" s="3" t="inlineStr"/>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>transfer(1)</t>
+        </is>
+      </c>
       <c r="D299" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5829,7 +7021,11 @@
           <t>storage</t>
         </is>
       </c>
-      <c r="C300" s="3" t="inlineStr"/>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>storage(3)</t>
+        </is>
+      </c>
       <c r="D300" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5847,7 +7043,11 @@
           <t>setup</t>
         </is>
       </c>
-      <c r="C301" s="3" t="inlineStr"/>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>setup(2)</t>
+        </is>
+      </c>
       <c r="D301" s="3" t="inlineStr">
         <is>
           <t>Original_300</t>
@@ -5999,7 +7199,7 @@
       </c>
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>conference(1)</t>
+          <t>conference(2)</t>
         </is>
       </c>
       <c r="D308" s="3" t="inlineStr">
@@ -6175,7 +7375,7 @@
       </c>
       <c r="C316" s="3" t="inlineStr">
         <is>
-          <t>pull(1), ups(1)</t>
+          <t>pull(2), ups(1)</t>
         </is>
       </c>
       <c r="D316" s="3" t="inlineStr">
@@ -6571,7 +7771,7 @@
       </c>
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>YouTube(1), season(1), finale(1)</t>
+          <t>YouTube(2), season(1), finale(1)</t>
         </is>
       </c>
       <c r="D334" s="3" t="inlineStr">
@@ -6791,7 +7991,7 @@
       </c>
       <c r="C344" s="3" t="inlineStr">
         <is>
-          <t>appraisal(1), budget(1)</t>
+          <t>appraisal(1), budget(2)</t>
         </is>
       </c>
       <c r="D344" s="3" t="inlineStr">
@@ -6835,7 +8035,7 @@
       </c>
       <c r="C346" s="3" t="inlineStr">
         <is>
-          <t>meeting(1)</t>
+          <t>meeting(3)</t>
         </is>
       </c>
       <c r="D346" s="3" t="inlineStr">
@@ -6945,7 +8145,7 @@
       </c>
       <c r="C351" s="3" t="inlineStr">
         <is>
-          <t>conference(2)</t>
+          <t>conference(3)</t>
         </is>
       </c>
       <c r="D351" s="3" t="inlineStr">
@@ -7429,7 +8629,7 @@
       </c>
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>deadline(1)</t>
+          <t>deadline(2)</t>
         </is>
       </c>
       <c r="D373" s="3" t="inlineStr">
@@ -7451,7 +8651,7 @@
       </c>
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>Netflix(1)</t>
+          <t>Netflix(3)</t>
         </is>
       </c>
       <c r="D374" s="3" t="inlineStr">
@@ -7495,7 +8695,7 @@
       </c>
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>presentation(1)</t>
+          <t>presentation(2)</t>
         </is>
       </c>
       <c r="D376" s="3" t="inlineStr">
@@ -7605,7 +8805,7 @@
       </c>
       <c r="C381" s="3" t="inlineStr">
         <is>
-          <t>Netflix(2)</t>
+          <t>Netflix(4)</t>
         </is>
       </c>
       <c r="D381" s="3" t="inlineStr">
@@ -7715,7 +8915,7 @@
       </c>
       <c r="C386" s="3" t="inlineStr">
         <is>
-          <t>meeting(2), teamwork(1)</t>
+          <t>meeting(4), teamwork(1)</t>
         </is>
       </c>
       <c r="D386" s="3" t="inlineStr">
@@ -7825,7 +9025,7 @@
       </c>
       <c r="C391" s="3" t="inlineStr">
         <is>
-          <t>presentation(2)</t>
+          <t>presentation(3)</t>
         </is>
       </c>
       <c r="D391" s="3" t="inlineStr">
@@ -8727,7 +9927,7 @@
       </c>
       <c r="C432" s="3" t="inlineStr">
         <is>
-          <t>budget(2)</t>
+          <t>budget(3)</t>
         </is>
       </c>
       <c r="D432" s="3" t="inlineStr">
@@ -8947,7 +10147,7 @@
       </c>
       <c r="C442" s="3" t="inlineStr">
         <is>
-          <t>onboarding(1)</t>
+          <t>onboarding(2)</t>
         </is>
       </c>
       <c r="D442" s="3" t="inlineStr">
@@ -9475,7 +10675,7 @@
       </c>
       <c r="C466" s="3" t="inlineStr">
         <is>
-          <t>pull(2), downs(1)</t>
+          <t>pull(3), downs(1)</t>
         </is>
       </c>
       <c r="D466" s="3" t="inlineStr">
@@ -9541,7 +10741,7 @@
       </c>
       <c r="C469" s="3" t="inlineStr">
         <is>
-          <t>meeting(3)</t>
+          <t>meeting(5)</t>
         </is>
       </c>
       <c r="D469" s="3" t="inlineStr">
@@ -9629,7 +10829,7 @@
       </c>
       <c r="C473" s="3" t="inlineStr">
         <is>
-          <t>Starbucks(1)</t>
+          <t>Starbucks(2)</t>
         </is>
       </c>
       <c r="D473" s="3" t="inlineStr">
@@ -9717,7 +10917,7 @@
       </c>
       <c r="C477" s="3" t="inlineStr">
         <is>
-          <t>budget(3)</t>
+          <t>budget(4)</t>
         </is>
       </c>
       <c r="D477" s="3" t="inlineStr">
@@ -9893,7 +11093,7 @@
       </c>
       <c r="C485" s="3" t="inlineStr">
         <is>
-          <t>Starbucks(2)</t>
+          <t>Starbucks(3)</t>
         </is>
       </c>
       <c r="D485" s="3" t="inlineStr">
@@ -10575,7 +11775,7 @@
       </c>
       <c r="C516" s="3" t="inlineStr">
         <is>
-          <t>presentation(3)</t>
+          <t>presentation(4)</t>
         </is>
       </c>
       <c r="D516" s="3" t="inlineStr">
@@ -10773,7 +11973,7 @@
       </c>
       <c r="C525" s="3" t="inlineStr">
         <is>
-          <t>feedback(1)</t>
+          <t>feedback(2)</t>
         </is>
       </c>
       <c r="D525" s="3" t="inlineStr">
@@ -10927,7 +12127,7 @@
       </c>
       <c r="C532" s="3" t="inlineStr">
         <is>
-          <t>streaming(1)</t>
+          <t>streaming(2)</t>
         </is>
       </c>
       <c r="D532" s="3" t="inlineStr">
@@ -11961,7 +13161,7 @@
       </c>
       <c r="C579" s="3" t="inlineStr">
         <is>
-          <t>email(1)</t>
+          <t>email(2)</t>
         </is>
       </c>
       <c r="D579" s="3" t="inlineStr">
@@ -12049,7 +13249,7 @@
       </c>
       <c r="C583" s="3" t="inlineStr">
         <is>
-          <t>feedback(2)</t>
+          <t>feedback(3)</t>
         </is>
       </c>
       <c r="D583" s="3" t="inlineStr">
@@ -12247,7 +13447,7 @@
       </c>
       <c r="C592" s="3" t="inlineStr">
         <is>
-          <t>warm(1), up(1), rows(1)</t>
+          <t>warm(1), up(2), rows(1)</t>
         </is>
       </c>
       <c r="D592" s="3" t="inlineStr">
@@ -12269,7 +13469,7 @@
       </c>
       <c r="C593" s="3" t="inlineStr">
         <is>
-          <t>Apple(1)</t>
+          <t>Apple(2)</t>
         </is>
       </c>
       <c r="D593" s="3" t="inlineStr">
@@ -13589,7 +14789,7 @@
       </c>
       <c r="C653" s="3" t="inlineStr">
         <is>
-          <t>invoice(1)</t>
+          <t>invoice(3)</t>
         </is>
       </c>
       <c r="D653" s="3" t="inlineStr">
@@ -13875,7 +15075,7 @@
       </c>
       <c r="C666" s="3" t="inlineStr">
         <is>
-          <t>YouTube(2)</t>
+          <t>YouTube(3)</t>
         </is>
       </c>
       <c r="D666" s="3" t="inlineStr">
@@ -14161,7 +15361,7 @@
       </c>
       <c r="C679" s="3" t="inlineStr">
         <is>
-          <t>warm(2), up(2), rows(3)</t>
+          <t>warm(2), up(3), rows(3)</t>
         </is>
       </c>
       <c r="D679" s="3" t="inlineStr">
@@ -14227,7 +15427,7 @@
       </c>
       <c r="C682" s="3" t="inlineStr">
         <is>
-          <t>Apple(2)</t>
+          <t>Apple(3)</t>
         </is>
       </c>
       <c r="D682" s="3" t="inlineStr">
@@ -14337,7 +15537,7 @@
       </c>
       <c r="C687" s="3" t="inlineStr">
         <is>
-          <t>email(2)</t>
+          <t>email(3)</t>
         </is>
       </c>
       <c r="D687" s="3" t="inlineStr">
@@ -14513,7 +15713,7 @@
       </c>
       <c r="C695" s="3" t="inlineStr">
         <is>
-          <t>cable(1), machine(1), warm(3), up(3)</t>
+          <t>cable(1), machine(1), warm(3), up(4)</t>
         </is>
       </c>
       <c r="D695" s="3" t="inlineStr">
@@ -14579,7 +15779,7 @@
       </c>
       <c r="C698" s="3" t="inlineStr">
         <is>
-          <t>invoice(2)</t>
+          <t>invoice(4)</t>
         </is>
       </c>
       <c r="D698" s="3" t="inlineStr">
@@ -14623,7 +15823,7 @@
       </c>
       <c r="C700" s="3" t="inlineStr">
         <is>
-          <t>presentation(4)</t>
+          <t>presentation(5)</t>
         </is>
       </c>
       <c r="D700" s="3" t="inlineStr">
@@ -14755,7 +15955,7 @@
       </c>
       <c r="C706" s="3" t="inlineStr">
         <is>
-          <t>email(3), deploy(1)</t>
+          <t>email(4), deploy(2)</t>
         </is>
       </c>
       <c r="D706" s="3" t="inlineStr">
@@ -14865,7 +16065,7 @@
       </c>
       <c r="C711" s="3" t="inlineStr">
         <is>
-          <t>Spotify(1)</t>
+          <t>Spotify(2)</t>
         </is>
       </c>
       <c r="D711" s="3" t="inlineStr">
@@ -15283,7 +16483,7 @@
       </c>
       <c r="C730" s="3" t="inlineStr">
         <is>
-          <t>conference(3)</t>
+          <t>conference(4)</t>
         </is>
       </c>
       <c r="D730" s="3" t="inlineStr">
@@ -16119,7 +17319,7 @@
       </c>
       <c r="C768" s="3" t="inlineStr">
         <is>
-          <t>conference(4)</t>
+          <t>conference(5)</t>
         </is>
       </c>
       <c r="D768" s="3" t="inlineStr">
@@ -16405,7 +17605,7 @@
       </c>
       <c r="C781" s="3" t="inlineStr">
         <is>
-          <t>pull(3), downs(2)</t>
+          <t>pull(4), downs(2)</t>
         </is>
       </c>
       <c r="D781" s="3" t="inlineStr">
@@ -16515,7 +17715,7 @@
       </c>
       <c r="C786" s="3" t="inlineStr">
         <is>
-          <t>pull(4), downs(3)</t>
+          <t>pull(5), downs(3)</t>
         </is>
       </c>
       <c r="D786" s="3" t="inlineStr">
@@ -16779,7 +17979,7 @@
       </c>
       <c r="C798" s="3" t="inlineStr">
         <is>
-          <t>Netflix(3)</t>
+          <t>Netflix(5)</t>
         </is>
       </c>
       <c r="D798" s="3" t="inlineStr">
@@ -16999,7 +18199,7 @@
       </c>
       <c r="C808" s="3" t="inlineStr">
         <is>
-          <t>trailer(3), Spotify(2)</t>
+          <t>trailer(3), Spotify(3)</t>
         </is>
       </c>
       <c r="D808" s="3" t="inlineStr">
@@ -17043,7 +18243,7 @@
       </c>
       <c r="C810" s="3" t="inlineStr">
         <is>
-          <t>presentation(5)</t>
+          <t>presentation(6)</t>
         </is>
       </c>
       <c r="D810" s="3" t="inlineStr">
@@ -17197,7 +18397,7 @@
       </c>
       <c r="C817" s="3" t="inlineStr">
         <is>
-          <t>deploy(2)</t>
+          <t>deploy(3)</t>
         </is>
       </c>
       <c r="D817" s="3" t="inlineStr">
@@ -17681,7 +18881,7 @@
       </c>
       <c r="C839" s="3" t="inlineStr">
         <is>
-          <t>pull(5), downs(4)</t>
+          <t>pull(6), downs(4)</t>
         </is>
       </c>
       <c r="D839" s="3" t="inlineStr">
@@ -17923,7 +19123,7 @@
       </c>
       <c r="C850" s="3" t="inlineStr">
         <is>
-          <t>Starbucks(3)</t>
+          <t>Starbucks(4)</t>
         </is>
       </c>
       <c r="D850" s="3" t="inlineStr">
@@ -18077,7 +19277,7 @@
       </c>
       <c r="C857" s="3" t="inlineStr">
         <is>
-          <t>conference(5)</t>
+          <t>conference(6)</t>
         </is>
       </c>
       <c r="D857" s="3" t="inlineStr">
@@ -18099,7 +19299,7 @@
       </c>
       <c r="C858" s="3" t="inlineStr">
         <is>
-          <t>meeting(4)</t>
+          <t>meeting(6)</t>
         </is>
       </c>
       <c r="D858" s="3" t="inlineStr">
@@ -18605,7 +19805,7 @@
       </c>
       <c r="C881" s="3" t="inlineStr">
         <is>
-          <t>meeting(5)</t>
+          <t>meeting(7)</t>
         </is>
       </c>
       <c r="D881" s="3" t="inlineStr">
@@ -19111,7 +20311,7 @@
       </c>
       <c r="C904" s="3" t="inlineStr">
         <is>
-          <t>Netflix(4)</t>
+          <t>Netflix(6)</t>
         </is>
       </c>
       <c r="D904" s="3" t="inlineStr">
@@ -19243,7 +20443,7 @@
       </c>
       <c r="C910" s="3" t="inlineStr">
         <is>
-          <t>invoice(3)</t>
+          <t>invoice(5)</t>
         </is>
       </c>
       <c r="D910" s="3" t="inlineStr">
@@ -19353,7 +20553,7 @@
       </c>
       <c r="C915" s="3" t="inlineStr">
         <is>
-          <t>resignation(1), feedback(3)</t>
+          <t>resignation(1), feedback(4)</t>
         </is>
       </c>
       <c r="D915" s="3" t="inlineStr">
@@ -19397,7 +20597,7 @@
       </c>
       <c r="C917" s="3" t="inlineStr">
         <is>
-          <t>report(1)</t>
+          <t>report(3)</t>
         </is>
       </c>
       <c r="D917" s="3" t="inlineStr">
@@ -19441,7 +20641,7 @@
       </c>
       <c r="C919" s="3" t="inlineStr">
         <is>
-          <t>warm(4), up(4)</t>
+          <t>warm(4), up(5)</t>
         </is>
       </c>
       <c r="D919" s="3" t="inlineStr">
@@ -19573,7 +20773,7 @@
       </c>
       <c r="C925" s="3" t="inlineStr">
         <is>
-          <t>networking(3), invoice(4)</t>
+          <t>networking(3), invoice(6)</t>
         </is>
       </c>
       <c r="D925" s="3" t="inlineStr">
@@ -19617,7 +20817,7 @@
       </c>
       <c r="C927" s="3" t="inlineStr">
         <is>
-          <t>deadline(2)</t>
+          <t>deadline(3)</t>
         </is>
       </c>
       <c r="D927" s="3" t="inlineStr">
@@ -19991,7 +21191,7 @@
       </c>
       <c r="C944" s="3" t="inlineStr">
         <is>
-          <t>email(4)</t>
+          <t>email(5)</t>
         </is>
       </c>
       <c r="D944" s="3" t="inlineStr">
@@ -20827,7 +22027,7 @@
       </c>
       <c r="C982" s="3" t="inlineStr">
         <is>
-          <t>report(2)</t>
+          <t>report(4)</t>
         </is>
       </c>
       <c r="D982" s="3" t="inlineStr">
@@ -20915,7 +22115,7 @@
       </c>
       <c r="C986" s="3" t="inlineStr">
         <is>
-          <t>streaming(2)</t>
+          <t>streaming(3)</t>
         </is>
       </c>
       <c r="D986" s="3" t="inlineStr">
@@ -20981,7 +22181,7 @@
       </c>
       <c r="C989" s="3" t="inlineStr">
         <is>
-          <t>Netflix(5)</t>
+          <t>Netflix(7)</t>
         </is>
       </c>
       <c r="D989" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Fix dialect purity issues and English/Arabic punctuation spacing
Per review feedback:
- Replaced "ضليت" (Levantine) with "قعدت" (Saudi) in 7 sentences.
- Replaced "صحابي" (Egyptian/Levantine) with "أصحابي" (Saudi) in 7 sentences.
- Added a space between Latin-script words and a following Arabic
  comma/exclamation mark (e.g. "checkout،" -> "checkout ،") across 39
  sentences, so TTS/ASR tokenization doesn't run the script boundary
  and the punctuation mark together.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155UPXv8Dk7askKg634TkFB
</commit_message>
<xml_diff>
--- a/arabic_english_codeswitching_1000_combined.xlsx
+++ b/arabic_english_codeswitching_1000_combined.xlsx
@@ -995,7 +995,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>الـ pipeline توقف بسبب خطأ في الـ config! لازم نصلحه الحين.</t>
+          <t>الـ pipeline توقف بسبب خطأ في الـ config ! لازم نصلحه الحين.</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1182,7 +1182,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>جرب تستخدم Postman عشان تختبر الـ API!</t>
+          <t>جرب تستخدم Postman عشان تختبر الـ API !</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -4038,7 +4038,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>وصلت لمرحلة الـ checkout، بس ليش الموقع يتوقف كل مرة؟</t>
+          <t>وصلت لمرحلة الـ checkout ، بس ليش الموقع يتوقف كل مرة؟</t>
         </is>
       </c>
       <c r="B213" s="3" t="inlineStr">
@@ -4786,7 +4786,7 @@
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>أرسلت له رسالة على WhatsApp، ليش ما رد لين الحين؟</t>
+          <t>أرسلت له رسالة على WhatsApp ، ليش ما رد لين الحين؟</t>
         </is>
       </c>
       <c r="B257" s="3" t="inlineStr">
@@ -5636,7 +5636,7 @@
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط Colours، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Colours ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B307" s="3" t="inlineStr">
@@ -5772,7 +5772,7 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>أختي ما تشتري مكياج إلا من MAC، وتقول الجودة تفرق عن أي ماركة ثانية.</t>
+          <t>أختي ما تشتري مكياج إلا من MAC ، وتقول الجودة تفرق عن أي ماركة ثانية.</t>
         </is>
       </c>
       <c r="B315" s="3" t="inlineStr">
@@ -6231,7 +6231,7 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في T4 وأنا في Tim Hortons، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في T4 وأنا في Tim Hortons ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B342" s="3" t="inlineStr">
@@ -6265,7 +6265,7 @@
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>كان عندي appraisal وبعده على طول budget، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
+          <t>كان عندي appraisal وبعده على طول budget ، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
         </is>
       </c>
       <c r="B344" s="3" t="inlineStr">
@@ -6350,7 +6350,7 @@
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Kart N Go، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Kart N Go ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B349" s="3" t="inlineStr">
@@ -6979,7 +6979,7 @@
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>كان عندي meeting وبعده على طول teamwork، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
+          <t>كان عندي meeting وبعده على طول teamwork ، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
         </is>
       </c>
       <c r="B386" s="3" t="inlineStr">
@@ -7336,7 +7336,7 @@
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>نزّلت sequel وبعدها series، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت sequel وبعدها series ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B407" s="3" t="inlineStr">
@@ -8152,7 +8152,7 @@
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Sudra Tea، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Sudra Tea ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B455" s="3" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط Avenues، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Avenues ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B460" s="3" t="inlineStr">
@@ -8254,7 +8254,7 @@
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>أختي ما تشتري مكياج إلا من Sephora، وتقول الجودة تفرق عن أي ماركة ثانية.</t>
+          <t>أختي ما تشتري مكياج إلا من Sephora ، وتقول الجودة تفرق عن أي ماركة ثانية.</t>
         </is>
       </c>
       <c r="B461" s="3" t="inlineStr">
@@ -8662,7 +8662,7 @@
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Starbucks، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Starbucks ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B485" s="3" t="inlineStr">
@@ -8696,7 +8696,7 @@
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>شاركت في تحدي cycling مع صحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
+          <t>شاركت في تحدي cycling مع أصحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
         </is>
       </c>
       <c r="B487" s="3" t="inlineStr">
@@ -9206,7 +9206,7 @@
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>شفت HBO الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت HBO الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B517" s="3" t="inlineStr">
@@ -9478,7 +9478,7 @@
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>شاركت في تحدي running مع صحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
+          <t>شاركت في تحدي running مع أصحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
         </is>
       </c>
       <c r="B533" s="3" t="inlineStr">
@@ -9546,7 +9546,7 @@
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>نزّلت HBO وبعدها soundtrack، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت HBO وبعدها soundtrack ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B537" s="3" t="inlineStr">
@@ -9563,7 +9563,7 @@
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>الفطور كان فيه ice cream sundae والعشاء steak، يوم أكل كامل ما نسيته بسهولة.</t>
+          <t>الفطور كان فيه ice cream sundae والعشاء steak ، يوم أكل كامل ما نسيته بسهولة.</t>
         </is>
       </c>
       <c r="B538" s="3" t="inlineStr">
@@ -9716,7 +9716,7 @@
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Ole، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Ole ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B547" s="3" t="inlineStr">
@@ -10175,7 +10175,7 @@
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>نزّلت rom-com وبعدها season finale، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت rom-com وبعدها season finale ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B574" s="3" t="inlineStr">
@@ -10311,7 +10311,7 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>شفت Shahid VIP الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت Shahid VIP الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B582" s="3" t="inlineStr">
@@ -10566,7 +10566,7 @@
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>الفطور كان فيه pasta والعشاء mac&amp;cheese، يوم أكل كامل ما نسيته بسهولة.</t>
+          <t>الفطور كان فيه pasta والعشاء mac&amp;cheese ، يوم أكل كامل ما نسيته بسهولة.</t>
         </is>
       </c>
       <c r="B597" s="3" t="inlineStr">
@@ -10940,7 +10940,7 @@
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في Lagate وأنا في City Fresh Kitchen، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في Lagate وأنا في City Fresh Kitchen ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B619" s="3" t="inlineStr">
@@ -10991,7 +10991,7 @@
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Costa، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Costa ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B622" s="3" t="inlineStr">
@@ -11450,7 +11450,7 @@
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>الفطور كان فيه bagel والعشاء iced coffee، يوم أكل كامل ما نسيته بسهولة.</t>
+          <t>الفطور كان فيه bagel والعشاء iced coffee ، يوم أكل كامل ما نسيته بسهولة.</t>
         </is>
       </c>
       <c r="B649" s="3" t="inlineStr">
@@ -11535,7 +11535,7 @@
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط Uptown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Uptown ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B654" s="3" t="inlineStr">
@@ -11739,7 +11739,7 @@
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>شفت YouTube الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت YouTube الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B666" s="3" t="inlineStr">
@@ -11756,7 +11756,7 @@
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>شفت prequel الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت prequel الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B667" s="3" t="inlineStr">
@@ -11824,7 +11824,7 @@
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط Boulevard World، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Boulevard World ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B671" s="3" t="inlineStr">
@@ -11909,7 +11909,7 @@
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>شاركت في تحدي taekwondo مع صحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
+          <t>شاركت في تحدي taekwondo مع أصحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
         </is>
       </c>
       <c r="B676" s="3" t="inlineStr">
@@ -12300,7 +12300,7 @@
     <row r="699">
       <c r="A699" s="2" t="inlineStr">
         <is>
-          <t>الفطور كان فيه hot chocolate والعشاء cupcake، يوم أكل كامل ما نسيته بسهولة.</t>
+          <t>الفطور كان فيه hot chocolate والعشاء cupcake ، يوم أكل كامل ما نسيته بسهولة.</t>
         </is>
       </c>
       <c r="B699" s="3" t="inlineStr">
@@ -12623,7 +12623,7 @@
     <row r="718">
       <c r="A718" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط Downtown، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط Downtown ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B718" s="3" t="inlineStr">
@@ -12810,7 +12810,7 @@
     <row r="729">
       <c r="A729" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في Lagate وأنا في Claro، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في Lagate وأنا في Claro ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B729" s="3" t="inlineStr">
@@ -13320,7 +13320,7 @@
     <row r="759">
       <c r="A759" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في Costa وأنا في Tim Hortons، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في Costa وأنا في Tim Hortons ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B759" s="3" t="inlineStr">
@@ -13592,7 +13592,7 @@
     <row r="775">
       <c r="A775" s="2" t="inlineStr">
         <is>
-          <t>الفطور كان فيه bubble tea والعشاء burrito، يوم أكل كامل ما نسيته بسهولة.</t>
+          <t>الفطور كان فيه bubble tea والعشاء burrito ، يوم أكل كامل ما نسيته بسهولة.</t>
         </is>
       </c>
       <c r="B775" s="3" t="inlineStr">
@@ -14153,7 +14153,7 @@
     <row r="808">
       <c r="A808" s="2" t="inlineStr">
         <is>
-          <t>نزّلت trailer وبعدها Spotify، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت trailer وبعدها Spotify ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B808" s="3" t="inlineStr">
@@ -14612,7 +14612,7 @@
     <row r="835">
       <c r="A835" s="2" t="inlineStr">
         <is>
-          <t>نزّلت Marvel وبعدها series، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت Marvel وبعدها series ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B835" s="3" t="inlineStr">
@@ -14935,7 +14935,7 @@
     <row r="854">
       <c r="A854" s="2" t="inlineStr">
         <is>
-          <t>شفت league حماسي أمس وانبسطت مرة، وقعدت أتكلم عنه مع صحابي طول اليوم.</t>
+          <t>شفت league حماسي أمس وانبسطت مرة، وقعدت أتكلم عنه مع أصحابي طول اليوم.</t>
         </is>
       </c>
       <c r="B854" s="3" t="inlineStr">
@@ -15037,7 +15037,7 @@
     <row r="860">
       <c r="A860" s="2" t="inlineStr">
         <is>
-          <t>شفت premiere الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت premiere الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B860" s="3" t="inlineStr">
@@ -15326,7 +15326,7 @@
     <row r="877">
       <c r="A877" s="2" t="inlineStr">
         <is>
-          <t>احتفلنا بتخرجها في مطعم وسط KAFD، وكانت الأمسية من أحلى الليالي هالسنة.</t>
+          <t>احتفلنا بتخرجها في مطعم وسط KAFD ، وكانت الأمسية من أحلى الليالي هالسنة.</t>
         </is>
       </c>
       <c r="B877" s="3" t="inlineStr">
@@ -15411,7 +15411,7 @@
     <row r="882">
       <c r="A882" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في T7 وأنا في Sudra Tea، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في T7 وأنا في Sudra Tea ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B882" s="3" t="inlineStr">
@@ -15649,7 +15649,7 @@
     <row r="896">
       <c r="A896" s="2" t="inlineStr">
         <is>
-          <t>شاركت في تحدي judo مع صحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
+          <t>شاركت في تحدي judo مع أصحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
         </is>
       </c>
       <c r="B896" s="3" t="inlineStr">
@@ -15666,7 +15666,7 @@
     <row r="897">
       <c r="A897" s="2" t="inlineStr">
         <is>
-          <t>زميلي مكتبه في 66 Cups وأنا في A5، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
+          <t>زميلي مكتبه في 66 Cups وأنا في A5 ، فنتقابل بس وقت الغدا لأن المسافة بينا بعيدة شوي.</t>
         </is>
       </c>
       <c r="B897" s="3" t="inlineStr">
@@ -15734,7 +15734,7 @@
     <row r="901">
       <c r="A901" s="2" t="inlineStr">
         <is>
-          <t>انصدمت من plot twist في الفيلم ولا توقعته أبدًا، وضليت أتكلم عنه مع صحابي كل الأسبوع.</t>
+          <t>انصدمت من plot twist في الفيلم ولا توقعته أبدًا، وقعدت أتكلم عنه مع أصحابي كل الأسبوع.</t>
         </is>
       </c>
       <c r="B901" s="3" t="inlineStr">
@@ -16142,7 +16142,7 @@
     <row r="925">
       <c r="A925" s="2" t="inlineStr">
         <is>
-          <t>كان عندي networking وبعده على طول invoice، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
+          <t>كان عندي networking وبعده على طول invoice ، يوم مرهق ما توقعت أخلصه بهالسرعة.</t>
         </is>
       </c>
       <c r="B925" s="3" t="inlineStr">
@@ -16159,7 +16159,7 @@
     <row r="926">
       <c r="A926" s="2" t="inlineStr">
         <is>
-          <t>نزّلت episode وبعدها animation، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
+          <t>نزّلت episode وبعدها animation ، قعدة سهر كاملة ما ندمت عليها أبدًا.</t>
         </is>
       </c>
       <c r="B926" s="3" t="inlineStr">
@@ -16227,7 +16227,7 @@
     <row r="930">
       <c r="A930" s="2" t="inlineStr">
         <is>
-          <t>شفت animation الجديد وصدمت من نهايته، وضليت أفكر فيه لين ثاني يوم.</t>
+          <t>شفت animation الجديد وصدمت من نهايته، وقعدت أفكر فيه لين ثاني يوم.</t>
         </is>
       </c>
       <c r="B930" s="3" t="inlineStr">
@@ -16720,7 +16720,7 @@
     <row r="959">
       <c r="A959" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في City Fresh Kitchen، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في City Fresh Kitchen ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B959" s="3" t="inlineStr">
@@ -17094,7 +17094,7 @@
     <row r="981">
       <c r="A981" s="2" t="inlineStr">
         <is>
-          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Chok، وقعدنا نضحك على مواقف الأسبوع.</t>
+          <t>احنا سوينا استراحة قصيرة وطلعنا نتغدى في Chok ، وقعدنا نضحك على مواقف الأسبوع.</t>
         </is>
       </c>
       <c r="B981" s="3" t="inlineStr">
@@ -17349,7 +17349,7 @@
     <row r="996">
       <c r="A996" s="2" t="inlineStr">
         <is>
-          <t>شاركت في تحدي boxing مع صحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
+          <t>شاركت في تحدي boxing مع أصحابي هالشهر، وكنا نتنافس على مين يلتزم أكثر.</t>
         </is>
       </c>
       <c r="B996" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Fix Egyptian dialect verb "عمل" family in the original 300 sentences
34 sentences used عملت/عملنا/نعمل/يعمل/أعمل ("did/make" in Egyptian
dialect) instead of the Saudi equivalent سويت/سوينا/نسوي/يسوي/أسوي.
Replaced all 34 with exact Saudi phrasing; left "العمل" (work/job),
"عملية" (transaction), and "عملاء" (customers) untouched since those
are standard nouns, not the dialect-marking verb. Also swept for other
Egyptian markers (تمام as standalone "okay", ازاي، مش، كده، إيه) --
none found; the "تمامًا" (completely) hits are standard MSA, not
dialect-specific, so left as-is. The new 700 file was already clean.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155UPXv8Dk7askKg634TkFB
</commit_message>
<xml_diff>
--- a/arabic_english_codeswitching_1000_combined.xlsx
+++ b/arabic_english_codeswitching_1000_combined.xlsx
@@ -621,7 +621,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>عملنا merge للـ branch في Git بعد المراجعة.</t>
+          <t>سوينا merge للـ branch في Git بعد المراجعة.</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -842,7 +842,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>الـ query بطيء لازم نعمل له optimize.</t>
+          <t>الـ query بطيء لازم نسوي له optimize.</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -876,7 +876,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>لازم نعمل test للـ feature قبل ما نطلعها.</t>
+          <t>لازم نسوي test للـ feature قبل ما نطلعها.</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -978,7 +978,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>عملنا setup لبيئة العمل على الـ cloud.</t>
+          <t>سوينا setup لبيئة العمل على الـ cloud.</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>لازم نعمل refactor للكود عشان يصير أنظف.</t>
+          <t>لازم نسوي refactor للكود عشان يصير أنظف.</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1250,7 +1250,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>عملت repost للـ tweet اللي عجبني.</t>
+          <t>سويت repost للـ tweet اللي عجبني.</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1352,7 +1352,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>عملت block لحساب مزعج على X.</t>
+          <t>سويت block لحساب مزعج على X.</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>عملت share للمنشور في الـ group.</t>
+          <t>سويت share للمنشور في الـ group.</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -1454,7 +1454,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>الحساب انعمله suspend بدون سبب واضح، للأسف!</t>
+          <t>صار على الحساب suspend بدون سبب واضح، للأسف!</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>عملت follow للحساب الجديد اللي فتحوه.</t>
+          <t>سويت follow للحساب الجديد اللي فتحوه.</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -1743,7 +1743,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>المؤثر عمل review صادق عن المنتج.</t>
+          <t>المؤثر سوى review صادق عن المنتج.</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>عملت subscribe لقناته الجديدة على YouTube.</t>
+          <t>سويت subscribe لقناته الجديدة على YouTube.</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -1879,7 +1879,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>عملنا collab مع حساب ثاني بنفس المجال.</t>
+          <t>سوينا collab مع حساب ثاني بنفس المجال.</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -2015,7 +2015,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>عملنا schedule لاجتماع الأسبوع الجاي.</t>
+          <t>سوينا schedule لاجتماع الأسبوع الجاي.</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -2100,7 +2100,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>عملت attach للملف قبل ما أرسل الإيميل.</t>
+          <t>سويت attach للملف قبل ما أرسل الإيميل.</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -2270,7 +2270,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>عملت approve على الطلب المالي.</t>
+          <t>سويت approve على الطلب المالي.</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -2644,7 +2644,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>لازم أعمل update للنظام قبل النوم.</t>
+          <t>لازم أسوي update للنظام قبل النوم.</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -2950,7 +2950,7 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>عملت sync بين الجوال واللابتوب.</t>
+          <t>سويت sync بين الجوال واللابتوب.</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -3171,7 +3171,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>الجوال دايم يعمل lag وقت فتح التطبيقات.</t>
+          <t>الجوال دايم يسوي lag وقت فتح التطبيقات.</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -3494,7 +3494,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>عملت subscription شهري لتطبيق التمارين.</t>
+          <t>سويت subscription شهري لتطبيق التمارين.</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -3919,7 +3919,7 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>عملت check-in مبكر عن طريق التطبيق.</t>
+          <t>سويت check-in مبكر عن طريق التطبيق.</t>
         </is>
       </c>
       <c r="B206" s="3" t="inlineStr">
@@ -4344,7 +4344,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>عملت refund للطلب لأنه تأخر كثير.</t>
+          <t>سويت refund للطلب لأنه تأخر كثير.</t>
         </is>
       </c>
       <c r="B231" s="3" t="inlineStr">
@@ -4463,7 +4463,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>عملت compare بين سعر المتجر والمتجر المنافس.</t>
+          <t>سويت compare بين سعر المتجر والمتجر المنافس.</t>
         </is>
       </c>
       <c r="B238" s="3" t="inlineStr">
@@ -4599,7 +4599,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>عملت order من تطبيق Jarir للأدوات المكتبية.</t>
+          <t>سويت order من تطبيق Jarir للأدوات المكتبية.</t>
         </is>
       </c>
       <c r="B246" s="3" t="inlineStr">
@@ -4854,7 +4854,7 @@
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>عملت install للتطبيق وواجهت مشكلة.</t>
+          <t>سويت install للتطبيق وواجهت مشكلة.</t>
         </is>
       </c>
       <c r="B261" s="3" t="inlineStr">
@@ -4905,7 +4905,7 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>عملت update للتطبيق عشان أحل المشكلة.</t>
+          <t>سويت update للتطبيق عشان أحل المشكلة.</t>
         </is>
       </c>
       <c r="B264" s="3" t="inlineStr">
@@ -4990,7 +4990,7 @@
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>عملت mute لمجموعة الواتساب المزعجة.</t>
+          <t>سويت mute لمجموعة الواتساب المزعجة.</t>
         </is>
       </c>
       <c r="B269" s="3" t="inlineStr">
@@ -5041,7 +5041,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>عملت forward للرسالة لصديقي.</t>
+          <t>سويت forward للرسالة لصديقي.</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>عملت clear للـ cache عشان يشتغل أسرع.</t>
+          <t>سويت clear للـ cache عشان يشتغل أسرع.</t>
         </is>
       </c>
       <c r="B280" s="3" t="inlineStr">
@@ -5262,7 +5262,7 @@
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>الجوال صار يعمل freeze بسبب كثرة التطبيقات.</t>
+          <t>الجوال صار يسوي freeze بسبب كثرة التطبيقات.</t>
         </is>
       </c>
       <c r="B285" s="3" t="inlineStr">
@@ -5279,7 +5279,7 @@
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>عملت restart سريع للجوال بعد ما تعلق.</t>
+          <t>سويت restart سريع للجوال بعد ما تعلق.</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
@@ -5347,7 +5347,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>عملت verify لرقمي بعد ما نزلت التطبيق.</t>
+          <t>سويت verify لرقمي بعد ما نزلت التطبيق.</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
@@ -5432,7 +5432,7 @@
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>عملت report لحساب مزيف يتصل بالناس.</t>
+          <t>سويت report لحساب مزيف يتصل بالناس.</t>
         </is>
       </c>
       <c r="B295" s="3" t="inlineStr">
@@ -5500,7 +5500,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>عملت transfer للملفات بين الجوالين بسرعة.</t>
+          <t>سويت transfer للملفات بين الجوالين بسرعة.</t>
         </is>
       </c>
       <c r="B299" s="3" t="inlineStr">

</xml_diff>